<commit_message>
fix: rename Col 5 header to Story IDs + correct UC-01/UC-04 status
- Col 5 header: "Trigger" → "Story IDs" (reflects actual content)
- UC-01 status: ✅ Done → ⚠️ Partial
- UC-04 status: ⚠️ Partial → ❌ Not Implemented
- Note: original Trigger column data was overwritten by Story IDs
  in previous commit; Trigger is not a Jira field and would need
  manual re-authoring if required

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/INTERNALCHATBOT_REQUIREMENTS_v5.xlsx
+++ b/INTERNALCHATBOT_REQUIREMENTS_v5.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Trigger</t>
+          <t>Story IDs</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>✅ Done</t>
+          <t>⚠️ Partial</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>⚠️ Partial</t>
+          <t>❌ Not Implemented</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix: rebuild UC summary sheet from scratch with correct 9-column layout
- Re-derived all data from Jira epics, agent-specs, and TEST_RECORD.md
- Correct columns: UC ID, UC Name, Description, Epic ID, Story IDs,
  Trigger, Acceptance Criteria, Implementation Status, Gap/Notes
- Story IDs now in Col 5, Trigger restored in Col 6
- Implementation Status corrected (UC-01: Partial, UC-04/UC-16: Not Implemented)
- Story Tracker sheet untouched

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/INTERNALCHATBOT_REQUIREMENTS_v5.xlsx
+++ b/INTERNALCHATBOT_REQUIREMENTS_v5.xlsx
@@ -482,17 +482,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -523,15 +524,20 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Trigger</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Implementation Status</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Gap/Notes</t>
         </is>
@@ -565,21 +571,121 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>1. Chatbot opens as embedded widget or page inside approved internal systems.
-2. User identity recognized via existing SSO/portal authentication (no re-login).
-3. User role (Student/Faculty/Staff) mapped from authentication context.
-4. Chatbot session starts on user trigger (click on button/widget/page).
-5. Chatbot respects role-based permissions throughout the session.</t>
+          <t>User opens an approved internal system/portal and clicks the chatbot widget or entry point.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>[UIB-1] Access chatbot widget from approved internal systems :
+1. The chatbot is available as an embedded widget (or page) within at least one approved internal system/portal/channel. 
+2. The list of “approved internal systems/portals/channels” is configurable (e.g., via admin configuration or environment settings). 
+3. The chatbot widget can be opened via: 
+* A visible “Chatbot” button/icon, or 
+* A dedicated chatbot section/page within the approved system. 
+4. When the user clicks on the chatbot button/icon: 
+* The chatbot widget opens within the same application context (e.g., side panel, modal, embedded frame, or dedicated page). 
+5. The chatbot widget: 
+* Loads successfully without requiring a separate username/password. 
+* Shows a default welcome message or greeting (configurable). 
+* Displays the user’s display name or a generic label (e.g., “Hi there”) based on available user info. 
+6. If the chatbot is accessed from a system/portal/channel that is not in the approved list: 
+* The chatbot widget does not load, 
+* And an appropriate error or fallback message is shown (e.g., “Chatbot not available in this application”). 
+7. The chatbot widget’s user interface is responsive and usable on: 
+* Desktop browsers 
+* Laptop screens 
+* (Optional) Mobile browser within the internal portal, if supported.
+[UIB-3] Seamless SSO-based access to chatbot:
+1. The chatbot relies on the existing organization authentication (SSO or portal authentication) and does not request a separate login screen for the user. 
+2. When an already authenticated user accesses the chatbot widget: 
+• The chatbot receives a valid, secure token or user context from the host system (e.g., SSO/portal). 
+• The chatbot uses that token/context to identify the user. 
+3. If the SSO/portal session is valid: 
+• The chatbot session is initialized automatically. 
+• The user can immediately start chatting without entering credentials. 
+4. If the SSO/portal session is not valid or has expired: 
+• The chatbot does not allow anonymous interaction (as per security policy). 
+• The chatbot shows a user-friendly message indicating that login is required via the host system (e.g., “Your session has expired. Please log in to the portal and try again.”). 
+5. At no point should the chatbot store or expose raw user passwords. 
+6. The chatbot must not expose sensitive authentication tokens in: 
+• UI 
+• Client-side logs 
+• Chat messages 
+7. The mechanism to verify SSO/portal authentication: 
+• Must use secure protocols (e.g., HTTPS) 
+• Must validate tokens/signatures (e.g., JWT validation, session validation) on the backend. 
+8. If there is an authentication error (e.g., invalid token, tampering detected): 
+• The chatbot session is not initialized. 
+• A generic error message is shown to the user (no internal technical details exposed). 
+9. SSO provider integrations
+• The SSO authentication mechanism supports integration with at least the following identity providers, using their standard protocols:
+ --&gt; Azure AD,
+ --&gt; Google,
+ --&gt; Generic SAML 2.0 identity providers,
+ --&gt; OAuth 2.0 / OIDC providers.
+• For each configured provider, the chatbot relies on the existing SSO/portal integration and does not introduce separate, duplicate login flows inside the chatbot.
+10. Audit logs &amp; auth observability
+• Authentication-related events relevant to chatbot access are logged on the backend for observability and audit, including at minimum:
+  --&gt; Login success / login failure for chatbot access,
+  --&gt;Role/persona assigned to the session (as determined in UIB‑10),
+  --&gt; Logout or session termination events where detectable.
+• These auth logs:
+  --&gt; Are not exposed in the chatbot UI, and
+  --&gt; Do not contain raw passwords or full tokens, but may contain safe identifiers (e.g., user ID, provider type, error codes) for troubleshooting.
+[UIB-10] Determine user persona from authentication context:
+1. Role/persona mapping configuration exists that defines: 
+• Supported personas: Student, Faculty, Staff. 
+• Mapping rules from SSO/portal attributes (e.g., groups, department codes, user type fields) to personas. 
+2. When a user opens the chatbot via an approved internal system: 
+• The chatbot backend reads role-relevant attributes from the SSO/portal context (e.g., claims, group memberships, user type fields). 
+3. The system evaluates mapping rules to determine the persona: 
+• If user meets “Student” criteria → persona is Student. 
+• If user meets “Faculty” criteria → persona is Faculty. 
+• If user meets “Staff” criteria → persona is Staff. 
+• The determined persona is attached to the chatbot session for that user. 
+4. If a user maps to multiple role rules: 
+• A clear precedence order is defined and configured (e.g., Faculty &gt; Staff &gt; Student), and 
+• The system applies this precedence consistently. 
+5. If the user does not match any configured role/persona rule: 
+• A default persona is applied (e.g., “Staff” or “Generic User”), 
+• Or access is denied based on configuration. 
+6. An admin can update role mapping rules without code change (e.g., via configuration file, admin UI, or environment variables). 
+7. Persona information should be accessible to: 
+• The chatbot logic (e.g., to define what content it can access). 
+• Any downstream services needing persona context (without exposing sensitive data). 
+• Persona information must not be editable by the end user from the chatbot UI.
+[UIB-14] Start chatbot interaction on user trigger:
+1. The chatbot session is initiated only after the user triggers one of the following: 
+• Clicks a “Chatbot” button/icon. 
+• Opens a dedicated chatbot page/section inside an approved system/portal/channel. 
+2. Upon trigger: 
+• The chatbot loads within a reasonable response time (e.g., configurable, such as under 3–5 seconds under normal network conditions). 
+• The user sees a visible loading indicator until the chatbot is ready for interaction. 
+3. The chatbot’s first view, once loaded, should: 
+• Display a welcome/greeting message (configurable). 
+• Indicate that the user is logged in (directly or implicitly; e.g., “Hi [First Name]” or “Welcome back.” if name is available). 
+4. Each new trigger should: 
+• Reuse an active session for the same authenticated user where applicable, or 
+• Start a new session based on configuration (e.g., after timeout). 
+5. If the session cannot be created due to backend errors: 
+• An appropriate error message is shown (e.g., “Unable to start chatbot right now. Please try again later.”). 
+• No partial or inconsistent UI is displayed. 
+6. Closing/minimizing the chatbot widget: 
+• Does not break the main host application. 
+• Optionally retains the conversation context if re-opened, based on configuration. 
+7. Security and privacy: 
+• Only the authenticated user can see their conversation. 
+• Conversation context is not visible to other users on the same device unless SSO/portal session is shared and permitted by policy.</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
           <t>⚠️ Partial</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Auth (JWT), login UI, role mapping implemented</t>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Auth (JWT) and login UI implemented; SSO integration and widget embedding not yet done</t>
         </is>
       </c>
     </row>
@@ -611,19 +717,109 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>1. User can submit natural-language queries without knowing specific system/document names.
-2. Chatbot searches only approved internal knowledge sources.
-3. Role/group-based permissions applied to filter search results.
-4. Response generated only from content user is authorized to see.
-5. Citations and links shown only for documents user can open.</t>
+          <t>User types a natural-language question into the chatbot and submits it.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
+          <t>[UIB-18] Submit a natural-language query:
+1. The chatbot shows an input field where the user can type a natural-language question.
+2. The user can submit a question by:
+• Pressing Enter, and/or
+• Clicking a visible “Send” or “Submit” button.
+3. After submission:
+• The question appears in the conversation as a user message.
+• The chatbot shows a clear indication that it is processing the query (e.g., typing/“Thinking…” indicator).
+• The chatbot accepts queries only from authenticated users (Students/Faculty/Staff) with a valid session.
+4. If the user’s session is invalid/expired:
+• The chatbot does not process the query, and
+• Shows a friendly message asking the user to log in again via the main portal/system.
+• Empty or blank messages are not sent (e.g., input with only spaces is blocked with a small validation message).
+5. Very long queries are handled safely:
+• Either accepted up to a maximum length, or
+• Rejected with a user-friendly message when they exceed the configured limit.
+[UIB-23] Retrieve from approved knowledge sources only:
+1. A configuration exists that defines which knowledge sources are “approved” (e.g., specific repos, KB spaces, internal portals).
+2. For every user query, the chatbot searches only within these approved knowledge sources.
+3. The chatbot does not use:
+• Unapproved internal repositories,
+• Public internet sources (unless explicitly allowed by configuration),
+• User content outside the approved list.
+4. Admins (or authorized roles) can update the list of approved sources without code change (e.g., configuration or admin UI).
+5. Any change to the list of approved sources is logged (who changed it, when, and what changed).
+6. If all approved sources are unavailable (e.g., outage):
+• The chatbot does not fall back to unapproved sources, and
+• Shows a friendly message (e.g., “I’m unable to access internal knowledge sources right now. Please try again later.”).
+7. No interpretation or recommendations
+• The chatbot does not provide legal, HR, or academic “advice”, and does not guess or fill gaps beyond what is explicitly in the authorized documents.
+• When content from authorized sources is unclear or conflicting, the chatbot presents the relevant sources or viewpoints neutrally, without choosing a side or recommending what the user should do.
+8. The restriction to approved sources is enforced in the backend, not only via UI.
+[UIB-27] Apply role/group-based permissions to filter results:
+1. For each authenticated session, the chatbot has access to the user’s role/persona (Student/Faculty/Staff) and, where available, group/permission attributes.
+2. When the chatbot searches approved knowledge sources:
+• It uses the user’s identity/permissions to filter which documents/records are visible to that user.
+3. Documents that the user does not have permission to access:
+• Are not returned in search results, and
+• Are not used for answer generation.
+• Source-system permissions (e.g., portal/KB/Confluence/Jira ACLs) are respected and not bypassed.
+• Additional chatbot-level rules (e.g., “Faculty-only content”, “Staff-only content”) can be configured and are applied consistently.
+4. If there is an error in checking permissions for a document:
+• The system treats that document as not accessible to the user (fail-safe).
+• Permission checks are implemented in the backend and cannot be bypassed by modifying the client/browser.
+[UIB-31] Generate response using only authorized content:
+1. The chatbot generates answers only from documents and records that:
+• Are in approved knowledge sources, and
+• Are allowed for the current user based on permissions.
+2. The chatbot must not:
+• Summarize content from documents the user cannot access, or
+• Reveal titles/snippets from restricted documents.
+3. If both authorized and unauthorized content match a query:
+• Only the authorized content is used to build the answer.
+• The chatbot does not indicate that extra restricted documents exist (no hints like “There are more documents you cannot access”).
+4. If no authorized content is found for the query:
+• The chatbot tells the user that it could not find information they have access to (using a friendly message).
+5. Any system error during answer generation (e.g., timeout, model error):
+• Shows a simple error message to the user, and
+• Still does not expose any restricted information.
+6. Logging/monitoring of answers does not include content from unauthorized documents.
+7. Concise, factual responses
+• The chatbot keeps answers short and to the point, avoiding unnecessary length when a concise response is sufficient.
+• Every statement in the answer is grounded only in the authorized, approved documents used for that response (as per criteria 1–3).
+8. Faithful summarization and paraphrasing
+• When summarizing or paraphrasing authorized content, the chatbot does not change the original meaning or introduce new facts that are not present in the underlying documents.
+• If the source content is ambiguous or conflicting, the chatbot either:
+   --&gt; Reflects that uncertainty clearly, or
+   --&gt; Follows the neutral / “no authorized information” pattern rather than inventing details.
+9. Source-aware, transparent answers
+• Each answer includes a sources section that shows, for every document used:
+ --&gt;  its name
+ --&gt; high-level location (repository/folder or space), and 
+ --&gt; version/date; 
+ --&gt; deep links are only shown for documents the user is authorized to access, 
+ --&gt; and no unauthorized documents appear in the sources list.
+[UIB-35] Provide citations and links only to authorized documents:
+1. When the chatbot adds citations or references in its answer:
+• Each citation refers only to a document/resource the user is allowed to access.
+2. Before showing each citation/link:
+• The system checks that the user has access to that specific document/resource.
+3. If the user does not have access to a document:
+• That document is not shown in the citations/links section.
+4. Citations should include:
+• A clear label (e.g., document title or source name, where allowed), and
+• A link that opens the document in its native internal system (e.g., portal/KB/Confluence).
+5. If documents used to generate the answer are not accessible to the user:
+• They are not listed in visible citations.
+6. If all potential sources for an answer are not accessible:
+• The chatbot does not show any links and instead uses the “no authorized information” behavior from UIB- 31: "Generate response using only authorized content"
+7. Citation format and behavior (e.g., inline numbers [1], [2], list at the end) can be configured.</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
           <t>✅ Done</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>RAG pipeline, RBAC filtering, citation extraction implemented</t>
         </is>
@@ -642,7 +838,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>This epic is about making sure the chatbot never exposes restricted documents or their details. When a user submits a query that matches restricted content, the chatbot must: Search only in approved sources. Return answers only from documents the user is allowed to see. Respond with a neutral message if no authorized documents are available. Never reveal restricted titles, locations, snippets, or the existence of restricted documents.</t>
+          <t>This epic is about making sure the chatbot never exposes restricted documents or their details. When a user submits a query that matches restricted content, the chatbot must search only in approved sources, return answers only from documents the user is allowed to see, respond with a neutral message if no authorized documents are available, and never reveal restricted titles, locations, snippets, or the existence of restricted documents.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -657,18 +853,88 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>1. Chatbot filters results to documents the user is authorized to access.
-2. Neutral response returned when only restricted documents match.
-3. Safe next steps optionally suggested when no accessible info found.
-4. Restricted document titles, locations, snippets, or existence never revealed.</t>
+          <t>User submits a query that matches restricted or access-controlled content.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
+          <t>[UIB-40] Filter to authorized documents only:
+1. For every query, the chatbot searches only in approved knowledge sources (as already defined in your “Retrieve from approved knowledge sources only” story, e.g., UIB‑23).
+2. For each matching document, the chatbot checks whether the current user (Student/Faculty/Staff) has permission to access that document.
+3. Documents that the user does not have access to:
+• Are removed from the candidate result set, and
+• Are not passed to answer generation.
+4. Documents the user is allowed to access:
+• Are kept as candidates for answer generation.
+5. The permission check uses:
+• Source system ACLs/permissions (portal/KB/Confluence/Jira/etc.), and/or
+• Chatbot-level role/group rules (e.g., “Faculty only”, “Staff only”).
+6. If a permission check for a document fails (error/timeout):
+• That document is treated as not accessible (fail-safe).
+• All filtering happens on the backend; the client cannot bypass it.
+7. Logging/monitoring does not store or expose lists of restricted document IDs/paths in a way visible to end users.
+[UIB-44] Neutral response when only restricted documents match:
+1. If a query matches only documents that are restricted for the user:
+• The chatbot does not generate an answer from those documents.
+2. In this case, the chatbot returns a neutral response such as:
+• “I couldn’t find information available to you on this topic.”
+3. The neutral response:
+• Does not mention that restricted documents exist.
+• Does not mention number, titles, or any details of restricted documents.
+4. If a query matches no documents at all (authorized or restricted):
+• The same or a similar neutral response is returned.
+• This behavior is consistent for all user types (Student, Faculty, Staff).
+5. System and error logs may record internal matching details for admins, but:
+• These details are not visible in the chatbot UI.
+6. Any model or backend error during this decision:
+• Must not cause restricted content to be used or hinted.
+• Should still result in a safe, neutral user message (possibly a generic error plus the “no info available to you” style).
+[UIB-48] Suggest safe next steps (optional, configurable):
+1. There is a configuration that controls whether “safe next steps” suggestions are enabled or disabled.
+2. Examples of safe next steps (configurable) may include:
+• “Contact the helpdesk at [email/phone].”
+• “Reach out to your department admin or supervisor.”
+• “Check the public FAQs or student handbook page.”
+3. When a query results in “no authorized documents” (as in  "Neutral response when only restricted documents match"):
+• If suggestions are enabled, the chatbot appends one or more safe suggestions below the neutral message.
+• If suggestions are disabled, only the neutral message is shown.
+4. Suggestions must not:
+• Include names, titles, or hints about restricted documents.
+• Point directly to restricted resources.
+• Suggestions can be managed without code change (e.g., configuration, admin UI, or content file).
+5. Different user roles (Student/Faculty/Staff) may have different suggestions (optional but allowed by design/config), e.g.:
+• Students → “Contact student support”
+• Faculty → “Contact academic support”
+6. If there is a configuration or loading error for suggestions:
+• The chatbot still returns the neutral response from  "Neutral response when only restricted documents match"
+• But silently omits next-step suggestions (no broken or partial text).
+[UIB-52] Do not reveal restricted titles, locations, snippets, or existence:
+1. For documents that the user is not authorized to access:
+• Titles are not shown anywhere in the chatbot UI.
+• Paths/URLs/locations are not shown.
+• Snippets or text excerpts are not shown.
+2. The chatbot does not:
+• Say “You don’t have access to document X.”
+• Indicate the number of restricted documents.
+• Describe restricted documents in any way (e.g., “There are HR policy docs you cannot see.”).
+3. In answers, citations, and any follow-up prompts:
+• Only authorized documents (for this user) can appear.
+• Any restricted document used internally must be completely hidden from the user-facing response.
+4. If a query strongly implies restricted content exists (for example, user guesses a restricted project name):
+• The chatbot still follows the neutral/no-authorized-info pattern (from Story 2) and does not confirm the existence of such content.
+5. Internal logs or admin views may show restricted matches for debugging, but:
+• These are never returned to the chatbot UI.
+• If there is any conflict between this rule and other features (e.g., retrieval, ranking), this rule wins:
+6. Restricted document details must never be exposed.
+7. Any new UI components (chips, suggestions, history, etc.) must also respect this rule and never reveal restricted document details.</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
           <t>✅ Done</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Two-layer RBAC enforcement (API route + chunk retrieval)</t>
         </is>
@@ -687,7 +953,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>This epic is about making sure the chatbot uses only the current, approved version of documents when answering user queries. When Admins enable governed 'current/approved' retrieval, the chatbot will: Use only the current, approved version from connected repositories. Ignore drafts, archived, or superseded versions based on configured rules. Show which version it used (document name + version/effective date + link).</t>
+          <t>This epic is about making sure the chatbot uses only the current, approved version of documents when answering user queries. When Admins enable governed 'current/approved' retrieval, the chatbot will use only the current approved version, ignore drafts/archived/superseded versions, and show which version it used.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -702,20 +968,95 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>1. Admin can enable governed 'current/approved' retrieval mode.
-2. Only current, approved document versions used in answers.
-3. Drafts, archived, and superseded versions ignored.
-4. Exact version cited (name + version/effective date + link).</t>
+          <t>Admin enables governed current/approved retrieval mode; user submits a query.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
+          <t>[UIB-57] Admin enables governed current/approved retrieval:
+1. There is a configuration or admin setting to enable or disable “current/approved retrieval” mode for the chatbot.
+2. When this mode is enabled:
+• The chatbot must use only documents marked as current/approved according to configured rules.
+3. When this mode is disabled:
+• The chatbot can use any accessible version.
+4. Admins can configure:
+• Which repositories or locations participate in governed current/approved retrieval.
+• Basic rules that distinguish current/approved content from drafts, archived or superseded versions (e.g., status, folder, metadata flags).
+5. Changes made by Admins (enable/disable, rule updates) are logged with:
+• Who changed it,
+• What changed,
+• When it changed.
+6. Configuration changes take effect for new queries without requiring a full deployment (e.g., reload from config on a schedule or via a light restart).
+7. If there is a configuration error or missing rules:
+• The chatbot must fail safe (either revert to a known default behavior or return a safe message),
+• And must not silently start using drafts or outdated documents as “current”.
+[UIB-61] Use only current, approved versions of documents:
+1. When governed current/approved retrieval is enabled (from UIB -57 ):
+• The chatbot only includes documents that meet the “current/approved” criteria for each repository.
+2. “Current/approved” criteria are based on configurable rules, for example:
+• A status field (e.g., Status = Approved),
+• A flag or label (e.g., current=true),
+• A specific path or folder (e.g., /Official, /Published).
+3. Drafts, archived, and superseded versions are excluded, such as:
+• Documents in Draft or Archive sections,
+• Earlier version numbers if a newer approved version exists,
+• Documents marked as “Deprecated”, “Superseded”, etc.
+4. The retrieval pipeline:
+• First filters by approved knowledge sources (UIB‑23),
+• Then filters by user access (UIB‑27, UIB‑40),
+• Then filters by current/approved version status (this story).
+5. If two or more documents conflict (e.g., same topic but different versions/states):
+• Only those marked as current/approved are used to generate the answer.
+6. If no “current/approved” version is available for a topic:
+• The chatbot does not fall back to drafts or archived versions,
+• And uses safe fallback behavior defined in UIB - 69.
+• This behavior applies consistently to all user types (Student, Faculty, Staff, Admin), subject to their existing access permissions.
+[UIB-65] Ignore drafts, archived, and superseded versions:
+1. The system can identify draft documents using repository-specific signals (e.g., draft status, draft folder, draft flag) and exclude them from:
+• Answer generation, and
+• Visible citations.
+2. The system can identify archived documents (e.g., archived folder, archive status) and exclude them in the same way.
+3. The system can detect superseded versions (e.g., version metadata indicates they are replaced by a newer approved version):
+• These superseded versions are not used for answering or citing.
+4. Admins can configure which metadata fields/values mean:
+• Draft,
+• Archived,
+• Superseded.
+5. If a document is mis‑labeled (e.g., a draft marked as approved):
+• The system still respects the configuration,
+• But such anomalies are visible in operational logs so admins can correct the source data.
+6. If a repository does not support explicit draft/archived/superseded flags:
+• Default rules can be configured (e.g., use only documents from certain folders/spaces considered “official”).
+7.  This ignoring behavior must not break or bypass document‑level access control and role filtering already defined (UIB‑27, UIB‑40, UIB‑52).
+[UIB-69] Cite exact version used (name + version/effective date + link):
+1. For each document used in answer generation:
+• The chatbot stores the specific version identifier (e.g., version number, revision ID, last updated / effective date).
+2. Citations in the chatbot’s response include, where available:
+• Document name or title,
+• Version identifier or effective date (e.g., “v3 – Effective from 01‑Jan‑2026”),
+• A link/URL that points to that exact version in the repository (or the canonical “current” view if version‑specific URLs are not supported).
+3. Citations follow existing authorization rules (from UIB‑35):
+• Only documents the user is allowed to access are cited.
+4. If the underlying repository supports version‑specific URLs:
+• The chatbot uses version‑specific URLs in citations.
+5. If the repository does not support version‑specific URLs:
+• The chatbot still includes version/effective date information in the label,
+• And links to the canonical document, clearly indicating the version used in the textual citation.
+6. If version metadata is missing or unclear for a document:
+*The chatbot either:
+--&gt; Omits that document from citations, or
+--&gt; Labels the citation in a way that does not falsely claim a specific version (e.g., “Policy Document (version unknown)”) based on configuration.
+7. Clicking a link should open the document in the native system (portal/KB/repo) where users can see the same version/content used for the answer (subject to that system’s own permissions).</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
           <t>❌ Not Implemented</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Basic retrieval works; version governance config not fully implemented</t>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Version governance config and draft/archive filtering not implemented</t>
         </is>
       </c>
     </row>
@@ -732,7 +1073,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>This epic defines how the chatbot behaves when more than one relevant document matches a user's query. The chatbot should: Collect multiple authorized, current documents. Consolidate insights from those documents into a clear answer. Cite multiple sources where applicable. Avoid confusion or leakage from restricted or outdated content.</t>
+          <t>This epic defines how the chatbot behaves when more than one relevant document matches a user's query. The chatbot should collect multiple authorized, current documents, consolidate insights into a clear answer, cite multiple sources where applicable, and avoid confusion or leakage from restricted or outdated content.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -747,21 +1088,74 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>1. All relevant, authorized, current documents collected for the query.
-2. Insights consolidated from multiple documents into one clear answer.
-3. Citations from multiple documents shown where applicable.
-4. Guidance provided when many documents are relevant (refine question).
-5. No confusion or leakage from restricted or outdated content.</t>
+          <t>User submits a query that matches more than one relevant, authorized document.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>⚠️ Partial</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Multi-doc retrieval via RAG; explicit consolidation UX not fully tested</t>
+          <t>[UIB-75] Aggregate multiple relevant documents:
+1. For each user query, after existing filters (approved sources, permissions, document-level access control, current/approved version rules) are applied: 
+• Only documents from approved sources are considered. 
+• Only documents the user is allowed to access are considered. 
+• Only current/approved versions are considered. 
+2. The retrieval layer can return a ranked list of multiple relevant documents (not just a single top result). 
+3. The maximum number of documents to consider (e.g., top N) is configurable. 
+4. Unauthorized, restricted, draft, archived, or superseded documents do not appear in the candidate list. 
+5. For each candidate document, the system stores: 
+• ID/URL, 
+• Title/name (where allowed), 
+• Relevance score, 
+• Version/effective date if available. 
+6. If only one document remains, it is still passed as a single-item list. 
+7. If no documents remain, existing “no authorized information” / neutral-response behavior is used (like UIB‑31 + UIB‑44).
+[UIB-79] Consolidate insights into one clear answer:
+1. When multiple documents are passed from retrieval, the answer-generation step can use several documents together as input. 
+2. The chatbot’s answer: 
+• Summarizes common points across documents clearly. 
+• Avoids repeating identical information from multiple sources. 
+3. The chatbot consolidates insights by: 
+• Combining consistent information into a single coherent explanation. 
+• Highlighting important variations only when needed (e.g., by program, campus, role). 
+4. If documents are broadly consistent, the chatbot returns a unified summary reflecting that consensus. 
+5. If documents differ or partially conflict: 
+• The chatbot clearly indicates differences (e.g., “For undergraduate programs…, for postgraduate programs…”). 
+• It does not expose restricted or outdated content. 
+6. All existing rules still apply: 
+• Authorized content only. 
+• No restricted titles/locations/snippets. 
+• Only current/approved versions. 
+7. Any LLM prompts for multi-document answers include only filtered, authorized, current documents (no restricted/superseded content).
+[UIB-83] Cite multiple sources where applicable:
+1. When an answer is based on more than one document, the chatbot includes multiple citations (e.g., [1], [2], [3]). 
+2. Each citation entry includes (where allowed): 
+• Document title/name, 
+• Version/effective date, 
+• Link to the document in its native system. 
+3. Only documents the user is allowed to access can appear as citations; restricted documents are never cited. 
+4. A sentence or paragraph can be associated with multiple citations (e.g., [1,2]) when insights come from multiple documents. 
+5. Documents used internally but not accessible to the user are not listed as citations. 
+6. If all underlying documents for an answer are inaccessible, the chatbot uses the “no authorized information” behavior and shows no links. 
+7. Clicking a citation link opens the document; if permissions change, the native system handles access, but the chatbot never intentionally links to an unauthorized document.
+[UIB-88] Help users when many documents are relevant:
+1. When the number of relevant, authorized, current documents exceeds a configurable threshold, the chatbot activates “many documents” behavior. 
+2. In this case, the chatbot can: 
+• Provide a concise high-level summary, and/or 
+• Ask clarifying questions to narrow the scope (e.g., year, program, campus, department). 
+3. Refinement suggestions are based only on documents the user is allowed to access and do not reveal restricted content. 
+4. Any implied counts or descriptions of “many documents” reflect only accessible documents. 
+5. The “many documents” threshold is configurable (not hard-coded). 
+6. When the user refines the query, the system reruns retrieval, consolidation, and citations for the refined query. 
+7. If “many documents” configuration fails, the chatbot falls back to a safe, conservative behavior (e.g., limit docs considered but still provide a clear consolidated answer with citations).</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Multi-doc retrieval and consolidation via RAG pipeline</t>
         </is>
       </c>
     </row>
@@ -793,16 +1187,42 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>1. Key details remembered within current session for follow-up questions.
-2. User can clear or reset context manually within a session.</t>
+          <t>User asks a follow-up or refinement question within the same chat session.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
+          <t>[UIB-93] Maintain context within an active session:
+1. For each user, the chatbot maintains a session context that includes: 
+• Recent user questions and chatbot answers. 
+• Key extracted parameters (e.g., course, term, campus, form type) when relevant. 
+2. Within an active session, the user can ask follow-up questions that rely on earlier information (e.g., “What about for next semester?”) and the chatbot correctly interprets them. 
+3. The chatbot uses context to: 
+• Resolve pronouns and references (“this course”, “that form”, “those dates”) when unambiguous. 
+• Maintain continuity over a short series of related questions. 
+4. Context is per user session and is not shared across different users. 
+5. If context becomes too long, the system: 
+• Uses a configured limit (e.g., last N turns or last M minutes) to keep only the most relevant parts. 
+6. Any personally identifiable or sensitive information stored in session context complies with institutional privacy and data-retention policies. 
+7. Admins can configure basic context-retention parameters (e.g., max turns, max time window).
+[UIB-98] Allow user to clear or reset context within a session :
+1. The chatbot UI includes an option to “Start new topic” / “Reset conversation” or similar control. 
+2. When the user chooses to reset: 
+• The chatbot stops using previous context for future answers. 
+• The user is clearly informed that a fresh context has started. 
+3. A new conversation context is created for the user without requiring them to log out. 
+4. Previous messages may still be visible in the UI history (depending on design), but are logically excluded from context used for new answers. 
+5. If the institution requires stronger privacy controls, an optional configuration can fully clear visible history on reset. 
+6. Reset is limited to the current user’s session and does not affect other users. 
+7. Any technical errors during reset result in a safe fallback (e.g., new context is created and user notified; no mixed-context behavior).</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
           <t>✅ Done</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Session-based context in agent.py</t>
         </is>
@@ -836,17 +1256,45 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>1. Context cleared when session expires or user logs out.
-2. Fresh context started on new session start.
-3. Old context does not carry over to new conversations.</t>
+          <t>User session expires, user logs out, or user starts a new session.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
+          <t>[UIB-103] Clear context when session expires or user logs out:
+1. The chatbot is tied to the institution’s session/auth system (portal/SSO). 
+2. When the underlying user session expires or the user logs out: 
+• The chatbot’s active session context for that user is marked as ended. 
+• Context from the ended session is not used for new queries. 
+3. If the user reopens the chatbot or logs in again: 
+• A fresh chatbot session is created with no carryover from previous context (unless explicit retention policy allows minimal non-personal history). 
+4. Any attempt to send a new query after expiration: 
+• Shows a message that the session has expired, and/or 
+• Prompts the user to log in again before continuing. 
+5. Admins can configure session timeout for chatbot independently or reuse institutional defaults (e.g., 30 minutes of inactivity). 
+6. Clearing context on expiry/log-out complies with privacy and institutional data policies. 
+7. Errors in detecting expiry or logout must fail safe (e.g., treat as expired and require re-authentication).
+[UIB-109] Start fresh context on new session start:
+1. When a user first opens the chatbot in a new authenticated session: 
+• A new chatbot conversation context is created. 
+2. The initial view of a new session: 
+• Shows a welcome/greeting message. 
+• Does not rely on any previous session’s questions/answers. 
+3. The system ensures that: 
+• Conversation contexts are correctly associated with session IDs or equivalent identifiers. 
+• One user’s past context is never incorrectly attached to another user’s new session. 
+4. If the system cannot safely determine whether a session is new: 
+• It treats it as new and does not reuse old context. 
+5. New session behavior is consistent for all roles (Student, Faculty, Staff, Admin). 
+6. Admins can optionally configure whether a small “last interaction summary” is shown or completely fresh start is always enforced.</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
           <t>✅ Done</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Session isolation in agent.py</t>
         </is>
@@ -880,17 +1328,42 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>1. Ambiguous or overly broad queries detected before answering.
-2. Chatbot asks user for clarification when query is unclear.
-3. More accurate answer provided after clarification.</t>
+          <t>User submits a query that is unclear, incomplete, or overly broad.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
+          <t>[UIB-113] Detect ambiguous or overly broad queries:
+1. The chatbot uses rules and/or model signals to identify: 
+• Queries that could refer to many different topics (e.g., “Tell me about exams”). 
+• Queries missing key parameters (e.g., “What is the fee?” without program/year). 
+• Queries that are vague (e.g., “Tell me everything about the university”). 
+2. A configurable set of patterns or heuristics helps detect such cases (e.g., generic nouns, long unstructured requests, missing required filters like program or semester). 
+3. The threshold for “too broad/ambiguous” is configurable. 
+4. The detection runs after permission and source checks to ensure restricted context isn’t used to guess user intent. 
+5. If detection fails, the chatbot still behaves safely (e.g., gives a cautious answer or a simple request for more detail). 
+6. Detection applies to all user roles (Student, Faculty, Staff, Admin).
+[UIB-117] Ask user for clarification before answering:
+1. When a query is flagged as ambiguous/broad: 
+• The chatbot does not attempt a detailed answer immediately. 
+• It responds with a clear, polite clarification prompt (e.g., “Can you specify which program or year you are asking about?”). 
+2. Clarification prompts may suggest options where appropriate (e.g., “Are you asking about [Undergraduate] or [Postgraduate] exams?”), but do not reveal any restricted details. 
+3. The user’s follow-up clarification is used to: 
+• Narrow the search space and improve relevance. 
+• Avoid unnecessary or irrelevant information. 
+4. If the user still responds vaguely: 
+• The chatbot may ask a second clarification or fall back to a safe high-level explanation. 
+• Clarification messages are consistent with institutional tone and can be configured. 
+5. Security and privacy are respected: clarification never exposes restricted titles/locations/snippets or confirms restricted content. 
+6. All interactions during clarification are logged (query, prompts, responses) for quality improvement, without including sensitive content in a way visible to end-users.</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
           <t>✅ Done</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Prompt-based clarification in ReAct agent template</t>
         </is>
@@ -924,17 +1397,39 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>1. Detected when no matching or authorized content exists.
-2. Safe fallback message returned instead of speculative answer.
-3. No guessing or invented answers.</t>
+          <t>User submits a query for which no matching or authorized content exists.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
+          <t>[UIB-123] Detect when no matching or authorized content exists:
+1. After searching approved sources and applying permission filters, the chatbot can determine when: 
+• No documents match the query at all, or 
+• Only restricted documents match (handled via your existing “neutral response” stories). 
+2. The detection logic is  implemented in the backend and cannot be bypassed from the UI. 
+3. The system differentiates between: 
+• “No content exists” vs 
+• “Content exists but not authorized” (to apply correct response logic). 
+4. Internal logs may record the distinction for admins, but this is not exposed to end-users. 
+5. Detection is consistent across all roles.
+[UIB-126] Return safe fallback instead of speculative answer:
+1. When no matching or authorized content exists for a query: 
+• The chatbot returns a clear fallback message (e.g., “I’m not able to find information on this topic in the university’s resources.”). 
+2. The chatbot does not: 
+• Invent facts or policies. 
+• Reference non-university sources unless explicitly allowed by policy. 
+3. The fallback message is configurable by admins to match institutional tone and guidelines. 
+4. The chatbot may optionally suggest safe next steps (if that separate use case is enabled), such as contacting support or visiting a general information page. 
+5. The fallback behavior is applied consistently across all roles. 
+6. Any technical error (e.g., search failure) is handled with a similarly safe message that does not expose system details or restricted content.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
           <t>✅ Done</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Fallback response logic in agent.py with retry</t>
         </is>
@@ -968,17 +1463,48 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>1. Unanswered queries logged with key metadata.
-2. Queries routed to designated university teams.
-3. Content gaps visible to administrators.</t>
+          <t>Chatbot cannot answer a user query after exhausting all retrieval attempts.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
+          <t>[UIB-131] Detect and log unanswered queries with metadata:
+1. An unanswered query is defined as: 
+• A query where the chatbot cannot provide a meaningful answer using available, authorized content, or 
+• A query explicitly flagged by the model/system as “low confidence” beyond a configured threshold. 
+2. For each unanswered query, the system logs at least: 
+• Query text (sanitized for privacy if necessary), 
+• User persona/role (Student/Faculty/Staff/Admin), 
+• Timestamp, 
+• Channel/portal where the question was asked, 
+• Optional: high-level category if determined. 
+3. Logs are stored in a secure, access-controlled repository compliant with university policies. 
+4. Sensitive or personal data is minimized/obfuscated according to data protection rules. 
+5. Logged items are clearly marked as “unanswered” or “low-confidence answers” for reporting. 
+6. Logging includes system errors that caused questions not to be answered.
+[UIB-135] Route unanswered queries to designated university teams:
+1. Admins can configure: 
+• Which team(s) receive unanswered queries (e.g., IT helpdesk, academic services, student support). 
+• The routing method (e.g., email, ticketing system, dashboard). 
+2. For each unanswered query, an escalation record is sent or created with: 
+• Query text, 
+• User persona/role, 
+• Timestamp and channel, 
+• Indication that it was unanswered/low-confidence. 
+3. Escalation targets can differ by: 
+• Persona (Student vs Faculty vs Staff), and/or 
+• Topic category (IT, academics, finance), if categorization is available. 
+• Escalation failures (e.g., email or ticket creation fails) are logged and visible to admins. 
+4. The system does not share restricted content or sensitive internal metadata in escalation messages; only safe and necessary details are included. 
+5. Teams can later use this information to improve content and chatbot behavior.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
           <t>✅ Done</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>DynamoDB escalation store + Slack webhook + admin endpoint (11 tests)</t>
         </is>
@@ -1012,19 +1538,43 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>1. Chatbot explains purpose and usage of institutional forms.
-2. Chatbot guides users on where to find forms.
-3. Answers based solely on documented information.</t>
+          <t>User asks about institutional forms (purpose, eligibility, location).</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>❌ Pending</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>No form-specific guidance implemented; handled by general RAG</t>
+          <t>[UIB-140] Answer questions about form purpose and usage:
+1. When a user asks about a form (e.g., “What is the leave application form for?”), the chatbot: 
+• Identifies the relevant form(s) using approved documentation. 
+2. The chatbot describes: 
+• The purpose of the form (what it is used for). 
+• Typical scenarios when it should be used. 
+• Any important eligibility or conditions noted in official documents. 
+3.  Information is strictly taken from approved institutional sources (no guesses). 
+4. If multiple forms are similar, the chatbot clarifies differences (e.g., “Form A is for staff; Form B is for students”). 
+5. If the form is not documented, the chatbot uses the “no matching content” behavior instead of inventing information. 
+6. Role-based differences (e.g., student vs faculty forms) are respected and explained where documented.
+[UIB-143] Guide users on where to find forms:
+1. For form-related queries, the chatbot can provide: 
+• Links or navigation paths to official form locations (e.g., portal pages, document repository, student information system). 
+2. Links are only provided to locations the user is allowed to access. 
+3.  If direct links cannot be provided (e.g., behind a different portal): 
+• The chatbot gives clear instructions on how to reach the form (e.g., “Log in to the portal, go to ‘Student Services’ &gt; ‘Forms’ &gt; ‘Leave Application’”). 
+4. Form locations are configured in a maintainable way (e.g., by admins in the Admin Console). 
+5. If a form location is missing or outdated, the chatbot: 
+• Avoids providing broken or guessed URLs. 
+• Can fall back to general guidance (e.g., “Please contact your program office for this form”). 
+6.  All links and instructions comply with access control rules.</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ Partial</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Handled by general RAG; no form-specific guidance logic</t>
         </is>
       </c>
     </row>
@@ -1056,19 +1606,43 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>1. Workflow-execution attempts detected.
-2. User informed that workflow execution is not supported.
-3. User directed to official systems for form submissions.</t>
+          <t>User attempts to submit, complete, or process a form/workflow via the chatbot.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>❌ Pending</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>No explicit workflow-prevention guardrail implemented</t>
+          <t>[UIB-148] Detect workflow-execution attempts:
+1. The chatbot recognizes requests that: 
+• Ask to submit or complete a form (e.g., “Submit my leave form”, “Apply for graduation now”). 
+• Ask to process approvals or make official changes (e.g., “Approve my registration”). 
+2. Detection uses: 
+• Keyword/intent rules (e.g., “submit”, “approve”, “apply now”). 
+• Optional model-based classification for workflow-like requests. 
+3. Detected workflow attempts are flagged internally but not executed. 
+4. Detection logic is configurable, so new patterns/phrases can be added. 
+5. Detected attempts are logged for future analysis, with appropriate privacy protections.
+[UIB-152] Inform users that workflow execution is not supported:
+1. When a workflow execution attempt is detected: 
+• The chatbot responds with a clear message (e.g., “I can’t submit or approve forms for you. Please use the official system or portal to complete this step.”). 
+2. The message: 
+• May include a link or instructions to the official system. 
+• Is configurable in tone and wording by admins. 
+3. The chatbot does not: 
+• Pretend that a form has been submitted. 
+• Partially fill or store form data as if submission is happening. 
+4. The chatbot can still provide informational guidance (from the “forms guidance” epic) alongside this message. 
+5. The behavior is consistent across all roles. 
+6. Workflow-execution attempts and the chatbot’s refusal are logged for audit and training.</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Handled via guardrails and agent prompt constraints</t>
         </is>
       </c>
     </row>
@@ -1100,17 +1674,40 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>1. Irrelevant or out-of-scope queries detected.
-2. Polite decline with scope guidance provided.
-3. Chatbot does not attempt to answer as general internet assistant.</t>
+          <t>User submits a query unrelated to institutional topics.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
+          <t>[UIB-157] Detect irrelevant or out-of-scope queries:
+1. The system identifies queries that: 
+• Are clearly outside university/institution domains (e.g., “Write my personal resume”, “What’s the weather tomorrow?”). 
+• Request general entertainment or non-educational content that is out-of-scope. 
+2. Detection uses: 
+• Keyword/domain rules, and/or 
+• Model-based classification for out-of-scope topics. 
+3. Boundaries of “in-scope” vs “out-of-scope” are defined and configurable by admins. 
+4. Detected irrelevant queries are not answered with domain-inaccurate guesses. 
+5. All detection is done server-side and cannot be bypassed via client modifications.
+[UIB-161] Provide polite decline and scope guidance:
+1. When a query is flagged as irrelevant/out-of-scope: 
+• The chatbot responds with a polite, short decline (e.g., “I’m here to help with information about this university, such as programs, policies, and services.”). 
+2. The message: 
+• Optionally includes examples of supported topics (e.g., “You can ask me about admissions, fees, academic policies, campus services…”). 
+• Is configurable by admins. 
+3. The chatbot does not: 
+• Attempt to answer the irrelevant query from external internet sources (unless explicitly allowed by policy). 
+• Generate inappropriate or harmful content. 
+4. The behavior is consistent across all roles. 
+5. Repeated irrelevant or abusive queries are passed to “Abuse &amp; Security Guardrails” behavior where applicable.</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
           <t>✅ Done</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Prompt-based handling in ReAct agent template</t>
         </is>
@@ -1144,17 +1741,53 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>1. Abusive or harmful queries detected.
-2. Blocked or safely responded to according to policy.
-3. Security events logged and optionally escalated.</t>
+          <t>User submits an abusive, harmful, or system-manipulation query.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
+          <t>[UIB-166] Detect abusive or harmful queries:
+1. The system detects: 
+• Abusive or harassing language. 
+• Self-harm, violence, or illegal activities. 
+• Attempts to circumvent permissions or extract restricted info (“jailbreak” attempts). 
+2. Detection methods include: 
+• Policy-based filters and keyword rules. 
+• Model-based classification for safety policy categories. 
+3. Admins can configure which categories are blocked vs. allowed with caution. 
+4. Detected queries are not processed as normal information requests. 
+5. Detection and classification decisions are logged (category, timestamp, anonymized user role if required).
+[UIB-170] Block or safely respond according to policy:
+1. For abusive content: 
+• The chatbot does not respond in kind. 
+• It returns a brief, policy-aligned message (e.g., “I can’t help with that kind of request.”). 
+2. For self-harm or severe risk content: 
+• The chatbot gives a compassionate, non-judgmental response. 
+• It may provide contact details for official university support or emergency services, consistent with policy. 
+3. For attempts to bypass permissions/manipulate system: 
+• The chatbot reiterates that it must follow institutional access and safety rules. 
+• It does not reveal restricted content or system internals. 
+4. Messages for each category are configurable and approved by the university. 
+5. Severe or repeated abuse/harm events can be flagged for admin review, if policy allows.
+[UIB-174] Log and optionally escalate security events:
+1. All guardrail-triggered events are logged with: 
+• Category (abuse, harm, manipulation, etc.), 
+• Timestamp, 
+• User role/persona (where allowed), 
+• Context needed for review (sanitized text, if allowed by policy). 
+2. Logs are stored securely and are accessible only to authorized staff. 
+3. Admins can configure: 
+• Which categories trigger an automatic escalation (e.g., email to security team, ticket creation). 
+4. Escalation messages do not include unnecessary personal data; they follow privacy guidelines. 
+5. Reporting and analytics can aggregate these events over time (counts, trends) without exposing individual identities improperly.</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
           <t>✅ Done</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>Two-layer guardrails (sync patterns + LLM classification), 27 tests</t>
         </is>
@@ -1188,17 +1821,43 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>1. Users can rate chatbot responses (thumbs up/down).
-2. Optional free-text feedback captured.
-3. Feedback recorded for analysis and quality improvement.</t>
+          <t>User clicks thumbs-up/thumbs-down on a chatbot response.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
+          <t>[UIB-179] Allow users to rate chatbot responses:
+1. Each chatbot answer includes an option to rate it (e.g., thumbs up/down, 1–5 stars). 
+2. Rating controls are simple and do not disrupt the conversation flow. 
+3. A rating by a user is associated with: 
+• The specific response, 
+• Timestamp, 
+• User role/persona (if allowed). 
+4. Users are not required to rate every response. 
+5. Ratings are stored in a secure data store and used only for improvement/analytics according to policy. 
+6. If the rating submission fails, the chatbot shows a small non-blocking error but conversation continues.
+[UIB-183] Capture optional free-text feedback:
+1. After rating, users can optionally: 
+• Add a short free-text comment. 
+2. Comments are associated with: 
+• The rating, 
+• The response ID, 
+• Timestamp, 
+• User role/persona (if permitted). 
+3. Length of comments is limited by configuration to prevent abuse. 
+4. Comments are stored securely and can be used by admins or content teams to: 
+• Identify common issues, 
+• Improve content and models. 
+5. Sensitive information in comments is discouraged (hint/messaging) and stored in compliance with privacy rules. 
+6. If comment submission fails, rating should still be preserved where possible.</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
           <t>✅ Done</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>DynamoDB feedback store + UI buttons + admin endpoint (12 tests)</t>
         </is>
@@ -1232,26 +1891,276 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>1. Role &amp; persona management configurable.
-2. Repository connector setup available.
-3. Indexing &amp; sync controls provided.
-4. Session &amp; experience controls configurable.
-5. Fallback &amp; user messaging configurable.
-6. Escalation routing &amp; notifications configurable.
-7. Branding &amp; UI theming configurable.
-8. Analytics &amp; logging dashboard available.
-9. Allowed file formats &amp; content processing configurable.
-10. Connector settings &amp; governance configurable.</t>
+          <t>Admin accesses the admin console to configure or monitor the chatbot.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>⚠️ Partial</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Admin API endpoints exist; full admin console UI not implemented</t>
+          <t>[UIB-188] Role &amp; Persona Management:
+1. Map identity groups to personas
+• Admin console provides a Role &amp; Persona Management screen.
+• Admin can define mapping rules from SSO/portal attributes (groups, department, user type) to personas: at least Student, Faculty, Staff, plus optional sub-groups (e.g., UG Student, PG Student).
+• These mappings are stored as configuration and are used by the runtime persona derivation story UIB‑10 – Determine user persona from authentication context.
+2. Assign document categories per persona
+• Admin can assign which high-level document categories (e.g., HR, Finance, IT, Academic, Research, Departmental) are visible per persona/sub-persona.
+• These category rules are applied alongside existing permission logic in UIB‑27 – Apply role/group-based permissions to filter results and UIB‑40 – Filter to authorized documents only.
+• Category rules cannot override source ACLs; they only further restrict or organise access.
+3. “Preview role permissions” for admins
+• Admin console allows selecting a persona (and optional sub-group) and running a “Preview what this role would see” simulation.
+• In preview mode, the system applies the configured persona/group and category rules (plus assumed standard permissions) and shows example:
+  --&gt; Accessible categories,
+  --&gt; Example documents or counts,
+  --&gt; Types of questions that would work.
+• Preview is clearly labelled as a simulation, not an actual user session, and does not expose any restricted document details that would violate UIB‑52.
+4. Configuration lifecycle and audit
+• Changes to persona mappings and document-category assignments:
+  --&gt; Take effect for new chatbot sessions (aligning with UIB‑10) without code deployment.
+ --&gt; Are recorded in an audit trail with admin ID, timestamp, and summary of changes.
+• If configuration is invalid (e.g., persona with no categories at all), the admin UI warns, and runtime fallbacks to safe defaults (e.g., minimal access) without breaking queries.
+[UIB-192] Repository Connector Setup:
+1. Connector catalog
+• Admin console shows a catalog of supported connector types:
+--&gt; SharePoint, OneDrive, Google Drive, LMS, File Server, Custom, etc.
+• Each connector type indicates:
+--&gt; Whether it is “Cloud” or “Drive” mode–capable.
+--&gt; Basic info (source system icon/name).
+2. Connector setup wizard
+• For each new connector, a step-by-step setup wizard is provided:
+--&gt; Step 1: Authentication/authorization (service account, app registration, credentials).
+--&gt; Step 2: Scope selection (sites/drives/libraries/folders).
+--&gt; Step 3: Basic options summary and test connection.
+• Successful completion creates a connector configuration that is referenced by runtime story UIB‑23 – Retrieve from approved knowledge sources only.
+3. Cloud vs Drive mode selection
+• Where applicable, the wizard allows selecting a mode:
+--&gt; Cloud (API-based remote access), or
+--&gt; Drive (local/sync-based access).
+• Mode is stored in connector config and drives how the backend connector (UIB‑24 – Backend connectors) behaves.
+4. Connector health page
+• For each configured connector, Admin Console shows a health view:
+  --&gt; Connection status (Connected / Error / Disabled).
+  --&gt; Last successful sync/index time.
+  --&gt; Last error message (admin-only detail).
+• Health information is read-only for standard admins and updated by backend processes; it doesn’t require a new deployment.
+[UIB-196] Indexing &amp; Sync Controls:
+1. Indexing type per connector 
+• For each connector, admin can choose indexing type: 
+  --&gt;Real-time / near real-time (if supported), or Batch. 
+ --&gt; The selected type is stored in configuration and used by the indexing pipeline (referenced by UIB‑24). 
+2. Batch frequency &amp; windows 
+• When Batch is selected, admin can configure: 
+ --&gt; Frequency: hourly/daily/weekly. 
+ --&gt; Optional allowed time windows (e.g., off-peak hours). 
+• These schedules control when indexing jobs are triggered; changing them does not require deployment. 
+3. View last run status 
+• For each connector, admin can view: 
+  --&gt; Last run start/end time, 
+  --&gt; Number of documents indexed/updated,    Number of failures/skipped items (e.g., format/size/permission). 
+• This status view is informational and supports troubleshooting when combined with existing logging stories (UIB‑23/27/31/40/44). 
+4. Manual “Run sync now” 
+• Admins with appropriate permission can click “Run sync now” for a connector. 
+• The system triggers an immediate indexing job respecting: 
+--&gt; Existing approved-sources configuration (UIB‑23), 
+--&gt; Permission and filtering rules (UIB‑27, UIB‑40). 
+• If a manual sync is already running, the UI clearly indicates this and prevents overlapping jobs or explains queued behaviour.
+[UIB-200] Session &amp; Experience Controls:
+1. Session timeout configuration 
+• Admin can configure chatbot session timeout duration (e.g., 15/30/60 mins) via Admin Console. 
+• This value is used by runtime behaviour described in UIB‑14 – Start chatbot interaction on user trigger (reuse vs new session after timeout). 
+2. Re-auth rules 
+• Admin can define re-auth rules, such as: 
+  --&gt;  Require re-authentication (via host SSO/portal) when session times out.
+  --&gt; Optionally require re-auth if critical persona/role attributes change during a session. 
+• These rules work within the existing SSO integration of UIB‑3 – Seamless SSO-based access to chatbot and do not introduce separate chatbot credentials. 
+3. Session reset behaviour 
+• Admin can set how the chatbot behaves when the user resets or starts a new session from the UI: 
+• Clear previous conversation context, or 
+Optionally show “recent history” if permitted. 
+• Closing/minimizing widget behaviour continues to follow UIB‑14 AC 6, but the admin-configured reset rules control what happens on explicit reset actions. 
+4. Safe defaults and audit 
+• If session configuration is missing or invalid, safe default values are applied (e.g., standard timeout). 
+• Changes to session settings are audit-logged with admin ID, timestamp, and new values, and apply to new sessions without code deployment.
+[UIB-204] Fallback &amp; User Messaging:
+1. Edit fallback messages 
+• Admin console provides editable text fields for: 
+  --&gt; No-match / “no relevant documents found” message. 
+ --&gt; Out-of-scope / “topic not covered” message. 
+ --&gt; Blocked/guardrail-hit message. 
+• These messages are used by runtime behaviours defined in UIB‑31, UIB‑44, and UIB‑48, instead of hard-coded text. 
+2. Clarification prompt style 
+• Admin can configure clarification prompt style, such as: 
+   --&gt; Whether to show short suggestion chips/buttons. 
+   --&gt; Maximum number of suggestions to display. 
+• Clarifiers do not reveal restricted content and remain consistent with no-leakage rules in UIB‑52. 
+3. Multi-language toggle (placeholder) 
+• A multi-language support toggle is available as a placeholder: 
+  --&gt; When off: only primary language messages are editable/used. 
+  --&gt;When on (future support), admin can view per-language placeholders or labels, even if runtime translation is not yet fully implemented. 
+• The toggle does not break existing behaviour and is clearly labelled as “future/limited support” if full localisation is not live. 
+4. Consistency &amp; audit 
+• Updated fallback texts and styles apply across all channels/pages where the chatbot is embedded (UIB‑1/14). 
+• All changes are tracked in an audit log (admin ID, time, before/after text).
+[UIB-208] Escalation Routing &amp; Notifications:
+1. Escalation destinations 
+• Admin can configure one or more destinations: 
+ --&gt; Email addresses (e.g., helpdesk, support team), 
+ --&gt; Helpdesk portal URL or ITSM ticket endpoint (if integrated). 
+ --&gt; Each destination has a label and type (email, URL/system). 
+2. Escalation rules 
+• Admin can configure which events trigger escalation, including: 
+  --&gt; Unanswered / “no authorized documents” outcomes (UIB‑44). 
+  --&gt; Repeated failures for the same user/session. 
+  --&gt; Very low feedback ratings (if feedback is available). 
+  --&gt;Guardrail hits (e.g., prompt injection, abusive queries) as defined by your guardrail logic. 
+• Rules can be enabled/disabled individually. 
+3. Metadata included in escalations 
+• Admin can define which metadata fields are included in an escalation payload, such as: 
+ --&gt; User persona (Student/Faculty/Staff), 
+ --&gt; Anonymised user identifier (if allowed), 
+ --&gt; User query or last few queries, 
+ --&gt;Sources attempted (at a high level—no restricted document IDs or paths). 
+• Metadata configuration must respect UIB‑52 – Do not reveal restricted titles, locations, snippets, or existence. 
+4. Test escalation flow 
+• From Admin Console, admin can click “Send test event” for a chosen rule/destination. 
+• A sample escalation is sent with clearly marked test content to confirm routing works (e.g., email received). 
+• Test flows are logged but do not affect production analytics or guardrail counts.
+[UIB-212] Branding &amp; UI Theming:
+1. Branding (logo &amp; colour) 
+• Admin can upload a logo (subject to file size/type limits) and choose primary theme colour(s). 
+• These branding settings apply consistently across chatbot surfaces (widget, full-page view) where applicable (UIB‑1 / UIB‑14). 
+2. UI component visibility 
+• Admin can control visibility of key UI components: 
+  --&gt; Citations panel (front-end representation of UIB‑35 behaviour), 
+  --&gt;Next-step suggestions panel (UI of UIB‑48 behaviour), 
+  --&gt;Feedback/ratings control (if present). 
+• Toggling visibility affects only presentation, not underlying guardrail behaviour (e.g., UIB‑35/48/52 still enforced even if UI is hidden). 
+3. Persona indicator toggle 
+• Admin can enable/disable a small persona indicator in the chatbot UI (e.g., “You are signed in as: Student”). 
+• When enabled, this indicator never shows raw group details or sensitive identifiers; it only shows persona labels derived from UIB‑10. 
+4. Widget embed settings 
+• Admin can configure: 
+  --&gt; Allowed embed domains/host applications (aligning with UIB‑1 – Access chatbot widget from approved internal systems). 
+  --&gt; Default widget placement (e.g., bottom-right floating, sidebar, full page) per host application type. 
+• Optional greeting behaviour (auto-greeting vs static state).
+[UIB-216] Analytics &amp; Logging Dashboard:
+1. Usage analytics 
+• Dashboard shows aggregate metrics for a selectable date range: 
+  --&gt; Total unique users, 
+  --&gt; Total sessions, 
+  --&gt; Total queries, 
+  --&gt;High-level trends over time (e.g., daily/weekly). 
+2. Popular queries &amp; topics 
+• Dashboard lists: 
+  --&gt; Top search queries, 
+  --&gt; Optionally clustered intents/topics or top departments/categories searched, based on available metadata. 
+• No restricted document details or contents are exposed in this view, consistent with UIB‑52. 
+3. Unanswered questions &amp; content gaps 
+• Dashboard shows: 
+  --&gt; “No match” / “no authorized documents” queries (from UIB‑44). 
+  --&gt; Repeated failures for similar queries. 
+• Content gaps view groups similar unanswered queries/themes to suggest where content is missing or outdated. 
+4. Guardrail hits 
+• Dashboard provides counts and trends for: 
+  --&gt; Prompt injection or policy-violating attempts (if detected), 
+  --&gt; Blocked/abusive queries, 
+  --&gt; Permission denials / restricted content matches. 
+• Only safe, anonymised information is displayed; no restricted titles/paths/snippets, following UIB‑52. 
+5. User satisfaction patterns 
+• Where feedback is present, the dashboard shows: 
+  --&gt; Rating distribution over time, 
+  --&gt; Low-rated topics, 
+  --&gt; Satisfaction by persona (Student/Faculty/Staff). 
+• Persona-level aggregation uses persona mapping rules from UIB‑10. 
+6. Filters &amp; drill-downs 
+• Admin can filter dashboard views by: 
+  --&gt; Date range, 
+  --&gt; Persona, 
+  --&gt; Department/category (if metadata exists), 
+  --&gt; Repository/source, 
+  --&gt; Channel (e.g., type of host application). 
+• Drill-downs allow viewing example queries or events under a metric without exposing restricted document details. 
+7. Export &amp; audit 
+• Admin can export selected analytics/log data as CSV or similar format. 
+• Export excludes sensitive document metadata and honours the no-leakage constraints from UIB‑31/40/52. 
+• Exports are logged (who exported what, when) for compliance.
+[UIB-482] Allowed File Formats &amp; Content Processing:
+1. Allowed file formats configuration exists 
+• The admin console provides a configuration area labelled “Allowed File Formats &amp; Content Processing”. 
+• It lists all supported file types (e.g., PDF, DOC/DOCX, XLS/XLSX, PPT/PPTX, TXT, image formats where applicable). 
+• For each type, the admin can enable or disable indexing via a toggle or checkbox. 
+2. Indexing respects allowed formats 
+• During indexing or sync, only files with enabled formats are processed and added to the chatbot index. 
+• Files with disabled formats are: 
+--&gt; Skipped from content extraction, and 
+--&gt; Logged as “skipped due to format rules” for admin/reporting, without causing indexing failure. 
+3. OCR toggle for images / scanned documents 
+• Where OCR is supported, the admin console exposes an “Enable OCR” setting for image/scanned PDF processing. 
+• When OCR is turned on: 
+--&gt; Text extraction from configured image/scanned formats is attempted during indexing. 
+• When OCR is turned off: 
+--&gt; Image/scanned files are not text-extracted for search; they are treated as unsupported content formats (and logged accordingly). 
+4. File size and page count limits 
+• Admins can set reasonable maximum file sizes and/or page counts to be processed (e.g., by connector or globally). 
+• Files exceeding these limits are not indexed and are logged as “skipped due to size/length limits”. 
+• Skipped items due to size/length do not break the indexing job; the overall job completes and records partial success. 
+5. Content processing rules for “final/approved only” 
+• Admins can define high-level content processing rules (for example, “Index only documents flagged as final/approved/published” where such metadata exists in the source system). 
+• When such a rule is active, drafts or non-approved versions are not indexed; only items meeting the rule are considered. 
+• The behaviour is consistent with existing “approved sources only” and “latest version” governance, and does not override document-level permissions. 
+6. Changes are configuration-only and audit-logged 
+• Changes to allowed formats, OCR settings, size/page limits, and content processing rules: 
+--&gt;Take effect on subsequent indexing runs (scheduled or manual) without requiring code deployment. 
+--&gt;Are logged with: admin identifier, date/time, and before/after values. 
+7. User-facing chatbot behaviour 
+• At query time, the chatbot only returns answers based on documents that have been successfully indexed under these rules (that is, in allowed formats and within limits). 
+• The chatbot does not mention skipped or unsupported files in user responses, maintaining the same neutrality and no-leakage principles as existing stories (e.g., UIB‑31, UIB‑44, UIB‑52).
+[UIB-487] Connector Settings &amp; Governance:
+1. Scope guardrails per connector 
+• For each configured connector, admin console exposes a “Scope &amp; Governance” section. 
+• Admins can define which sites/drives/libraries/folders are in scope for indexing (e.g., via selection UI or path patterns). 
+• Only items within these approved scopes are considered during indexing; any content outside scope is ignored and logged as “out-of-scope”. 
+• Scope rules are evaluated in the backend and cannot be bypassed from UI or runtime prompts. 
+2. Version control rules 
+• For each connector (or globally, where appropriate), admins can choose at least: 
+--&gt; “Index latest approved version only”, and 
+--&gt; “Include older versions only when explicitly requested” (future behaviour if implemented). 
+• When “latest-only” is selected: 
+--&gt; Indexing flags or selects the most recent approved version per document according to the source system’s version metadata. 
+--&gt; Superseded or archived versions are not used for primary answer generation. 
+• These rules are consistent with the “Retrieve Latest Document Version” behaviour already defined for runtime (they govern what goes into the index). 
+3. Metadata retention rules 
+• Admins can define retention policies for indexed metadata (for example, how long index entries and associated logs are retained). 
+• The retention settings are applied by housekeeping processes that remove or anonymize old index metadata and logs after the defined period. 
+• Retention policies are independent from the source system’s own content retention (the chatbot does not delete source documents). 
+4. Connector-level governance settings do not relax permissions 
+• Scope and version rules cannot override or weaken source system permissions (as defined in stories like UIB‑23, UIB‑27, UIB‑40). 
+• Even if a path is in-scope, document-level ACLs must still be respected at indexing and query time. 
+• Admin UI clearly indicates that governance settings are additive constraints, not substitutes for source access control. 
+5. Configuration changes apply without deployment 
+• Updates to connector scope, version rules, and retention settings are implemented as configuration data. 
+• New settings apply on subsequent indexing/sync runs (scheduled or manual) for each connector. 
+• No application deployment or code change is required for these governance adjustments. 
+6. Audit log for connector governance changes 
+• Each connector’s “Scope &amp; Governance” section surfaces an audit log of changes, including: 
+--&gt; Admin identifier who made the change. 
+--&gt; Timestamp. 
+--&gt; Summary of changes (e.g., “Added site X; removed folder Y; version rule changed from A to B; retention from 90 to 180 days”). 
+• The audit log is read-only to regular admins and cannot be edited via the UI. 
+• Log entries are stored according to the overall logging/retention policies defined for the chatbot. 
+7. Resilience and safe failure 
+• If connector governance configuration is invalid (e.g., all scopes removed or misconfigured): 
+--&gt; Indexing for that connector fails gracefully with clear admin-visible errors. 
+--&gt; No unintended or out-of-scope content is indexed. 
+• The chatbot continues to serve content from other healthy connectors and previously indexed data where appropriate, consistent with existing “approved sources only” behaviour.</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>❌ Not Implemented</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Admin API has document CRUD only; full admin console not implemented</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: UC-11 form guidance — UIB-140 + UIB-143
UIB-140 (Answer questions about form purpose):
- AC coverage: 6/6 criteria met
- System prompt updated with form identification + guidance behavior
- Tests added: 6 (tagged UIB-140-AC1 through AC6)

UIB-143 (Guide users on where to find forms):
- AC coverage: 5/6 (AC4 blocked on UC-16 Admin Console)
- System prompt extended with location guidance behavior
- Tests added: 5 (tagged UIB-143-AC1,2,3,5,6)
- CONFLICTS.md: UIB-143-AC4 logged as blocked

Regression: all 150 tests passing
Spec updated: agent-specs/05_AGENT.md

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/INTERNALCHATBOT_REQUIREMENTS_v5.xlsx
+++ b/INTERNALCHATBOT_REQUIREMENTS_v5.xlsx
@@ -1574,7 +1574,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Handled by general RAG; no form-specific guidance logic</t>
+          <t>UIB-140: 6/6 AC done, 6 tests. UIB-143: 5/6 AC done (AC4 blocked on UC-16), 5 tests. System prompt updated with form guidance + location guidance.</t>
         </is>
       </c>
     </row>
@@ -3994,11 +3994,11 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Partial</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="H33" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I33" s="5" t="inlineStr"/>
     </row>
@@ -4044,11 +4044,11 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Partial</t>
+          <t>⚠️ Partial (AC4 blocked on UC-16)</t>
         </is>
       </c>
       <c r="H34" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I34" s="2" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
fix: RBAC citation filter — post-generation source filtering
Root cause: _extract_sources() returned all sources with zero
role validation, leaking restricted document names to
unauthorized users even when answer content was correct.

Fix: _filter_sources_by_role() inserted in chat() between
source extraction and response return. Checks each cited
filename against allowed_roles from DynamoDB metadata.
Fallback/neutral responses now always return empty sources [].

Resolves: UIB-31, UIB-35, UIB-40, UIB-44, UIB-52
Tests added: 6 (TestRBACCitationFilter)
Regression: all 156 tests passing
Spec updated: agent-specs/05_AGENT.md

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/INTERNALCHATBOT_REQUIREMENTS_v5.xlsx
+++ b/INTERNALCHATBOT_REQUIREMENTS_v5.xlsx
@@ -2719,7 +2719,7 @@
         </is>
       </c>
       <c r="H9" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I9" s="5" t="inlineStr"/>
     </row>
@@ -2773,7 +2773,7 @@
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
     </row>
@@ -2827,7 +2827,7 @@
         </is>
       </c>
       <c r="H11" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I11" s="5" t="inlineStr"/>
     </row>
@@ -2882,7 +2882,7 @@
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
     </row>
@@ -2998,7 +2998,7 @@
         </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
feat: UC-12 workflow prevention + citation format enrichment (M1/UIB-35)
UC-12 (UIB-148 + UIB-152): Add workflow_guard.py with regex-based
detection of submit/approve/process/enroll attempts. Intercepts in
chat_router before agent runs, returns configurable refusal message.
Patterns configurable via WORKFLOW_PATTERNS env var. Escalation logged.
17 tests added (test_workflow_guard.py).

M1/UIB-35: Enrich SourceDoc with display_name and uploaded_at from
DynamoDB metadata. _enrich_sources() populates fields post-extraction.
Frontend shows display name instead of raw filename, shows upload date.
7 tests added (TestCitationFormatUC02).

186 tests passing (169 + 17 UC-12).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/INTERNALCHATBOT_REQUIREMENTS_v5.xlsx
+++ b/INTERNALCHATBOT_REQUIREMENTS_v5.xlsx
@@ -2773,9 +2773,13 @@
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="I10" s="2" t="inlineStr"/>
+        <v>13</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>RBAC filter (6 tests) + citation format enrichment with display_name/uploaded_at (7 tests)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: update Epic-Story implementation status from code evidence
Story Tracker: all 52 stories re-verified against codebase
- grep -rn "# AC: UIB-" used for exact AC-tag counts
- Code existence verified per story via agent exploration
- 6 status corrections: UIB-1 (Done→Partial), UIB-3 (Done→Pending),
  UIB-48 (Done→Pending), UC-04 all (Partial→Pending),
  UC-08 (Done→Partial), UIB-212 (Partial→Pending)

UC Summary: status derived from child story statuses
Tests Tagged: updated from actual grep counts (51 AC-tagged)
Source of truth: code + tagged tests, not assumptions

Totals: 31 Done, 9 Partial, 12 Pending | 193 tests passing

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/INTERNALCHATBOT_REQUIREMENTS_v5.xlsx
+++ b/INTERNALCHATBOT_REQUIREMENTS_v5.xlsx
@@ -685,7 +685,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Auth (JWT) and login UI implemented; SSO integration and widget embedding not yet done</t>
+          <t>UIB-10,UIB-14 done. UIB-1 partial (standalone app, not widget). UIB-3 pending (no SSO).</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>RAG pipeline, RBAC filtering, citation extraction implemented</t>
+          <t>RAG pipeline, RBAC filtering, citation enrichment all implemented. 11 AC-tagged tests.</t>
         </is>
       </c>
     </row>
@@ -931,12 +931,12 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>✅ Done</t>
+          <t>⚠️ Partial</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Two-layer RBAC enforcement (API route + chunk retrieval)</t>
+          <t>UIB-40,44,52 done. UIB-48 pending — no configurable next-step suggestions (Gap M7).</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Version governance config and draft/archive filtering not implemented</t>
+          <t>No version governance, draft/archived status, or version citations.</t>
         </is>
       </c>
     </row>
@@ -1150,12 +1150,12 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>✅ Done</t>
+          <t>⚠️ Partial</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Multi-doc retrieval and consolidation via RAG pipeline</t>
+          <t>RAG retriever_top_k=5 returns multi-doc. No explicit aggregation UX or disambiguation. No tests.</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Session-based context in agent.py</t>
+          <t>Session memory + TTL cleanup. 6 AC-tagged tests.</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Session isolation in agent.py</t>
+          <t>TTL-based expiry + fresh session on new ID.</t>
         </is>
       </c>
     </row>
@@ -1360,12 +1360,12 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>✅ Done</t>
+          <t>⚠️ Partial</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Prompt-based clarification in ReAct agent template</t>
+          <t>Prompt template has CLARIFICATION section but clarify_ambiguous_prompt defaults to empty.</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Fallback response logic in agent.py with retry</t>
+          <t>Fallback detection + safe response + FAISS last resort.</t>
         </is>
       </c>
     </row>
@@ -1506,7 +1506,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>DynamoDB escalation store + Slack webhook + admin endpoint (11 tests)</t>
+          <t>DynamoDB escalation store + Slack webhook. 11 tests (no AC tags).</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>UIB-140: 6/6 AC done, 6 tests. UIB-143: 5/6 AC done (AC4 blocked on UC-16), 5 tests. System prompt updated with form guidance + location guidance.</t>
+          <t>UIB-140: 6/6 AC done, 6 tests. UIB-143: 5/6 AC done (AC4 blocked on UC-16), 5 tests.</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Handled via guardrails and agent prompt constraints</t>
+          <t>workflow_guard.py + chat_router interception. 17 AC-tagged tests.</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Prompt-based handling in ReAct agent template</t>
+          <t>Prompt-based detection + configurable decline message.</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Two-layer guardrails (sync patterns + LLM classification), 27 tests</t>
+          <t>Two-layer guardrails (sync patterns + LLM). 27 tests (no AC tags).</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>DynamoDB feedback store + UI buttons + admin endpoint (12 tests)</t>
+          <t>DynamoDB feedback store + POST /feedback. 12 tests (no AC tags).</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Admin API has document CRUD only; full admin console not implemented</t>
+          <t>Only document CRUD admin API. 9/10 stories pending. Full admin console not built.</t>
         </is>
       </c>
     </row>
@@ -2292,7 +2292,11 @@
       <c r="H2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Frontend exists as standalone React app, not embeddable widget. No SSO integration.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -2362,13 +2366,17 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Partial</t>
+          <t>❌ Pending</t>
         </is>
       </c>
       <c r="H3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I3" s="5" t="inlineStr"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>No SSO/SAML/LDAP. JWT + local SQLite users.db only.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2423,13 +2431,17 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Partial</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Role extracted from JWT in decode_token(). Passed as Role enum to agent.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2484,13 +2496,17 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Partial</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="H5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="5" t="inlineStr"/>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Frontend ChatInput + New Chat button trigger chat interaction.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2545,7 +2561,11 @@
       <c r="H6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>POST /chat endpoint in chat_router.py. Frontend sends via useChat hook.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2600,7 +2620,11 @@
       <c r="H7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I7" s="5" t="inlineStr"/>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>tools.py filters by allowed_roles. document_store only returns INGESTED docs.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2651,7 +2675,11 @@
       <c r="H8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>_filter_by_role() in tools.py. OData filter for Azure, client-side for FAISS.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -2719,9 +2747,13 @@
         </is>
       </c>
       <c r="H9" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I9" s="5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>_filter_sources_by_role() post-generation RBAC filter in agent.py.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2773,11 +2805,11 @@
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>RBAC filter (6 tests) + citation format enrichment with display_name/uploaded_at (7 tests)</t>
+          <t>RBAC citation filter (1 tag) + enrichment with display_name/uploaded_at (9 tags).</t>
         </is>
       </c>
     </row>
@@ -2831,9 +2863,13 @@
         </is>
       </c>
       <c r="H11" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I11" s="5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>_filter_by_role() + OData filter. Search-layer + citation-layer RBAC.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2886,9 +2922,13 @@
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Fallback with _has_sources() returns sources:[]. UIB-44 tag in tests.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -2940,13 +2980,17 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>✅ Done</t>
+          <t>❌ Pending</t>
         </is>
       </c>
       <c r="H13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I13" s="5" t="inlineStr"/>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>No configurable next-step suggestions. Static fallback message only. Gap M7.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3002,9 +3046,13 @@
         </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="I14" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>_filter_sources_by_role() strips restricted docs from citations.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -3060,7 +3108,11 @@
       <c r="H15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I15" s="5" t="inlineStr"/>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>No version governance config. No approval workflow.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3120,7 +3172,11 @@
       <c r="H16" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>No version field in document metadata. All INGESTED docs treated equally.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -3176,7 +3232,11 @@
       <c r="H17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I17" s="5" t="inlineStr"/>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>No DRAFT/ARCHIVED status in document_store.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3234,7 +3294,11 @@
       <c r="H18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>No version/date field in SourceDoc beyond uploaded_at.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -3282,13 +3346,17 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>✅ Done</t>
+          <t>⚠️ Partial</t>
         </is>
       </c>
       <c r="H19" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I19" s="5" t="inlineStr"/>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>RAG retriever_top_k=5 returns multi-doc chunks. No explicit aggregation logic.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3338,13 +3406,17 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>✅ Done</t>
+          <t>⚠️ Partial</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Prompt says 'summarise'. No structured consolidation post-processing.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -3388,13 +3460,17 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>✅ Done</t>
+          <t>⚠️ Partial</t>
         </is>
       </c>
       <c r="H21" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I21" s="5" t="inlineStr"/>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>_extract_sources() parses multiple sources. No tagged tests.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3437,13 +3513,17 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>✅ Done</t>
+          <t>❌ Pending</t>
         </is>
       </c>
       <c r="H22" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>No disambiguation or guidance when many docs match.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -3495,7 +3575,11 @@
       <c r="H23" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="I23" s="5" t="inlineStr"/>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>ConversationBufferWindowMemory(k=10). TTL cleanup. 6 tagged tests.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3544,7 +3628,11 @@
       <c r="H24" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>clear_session() + POST /chat/clear. Frontend New Chat button.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -3596,7 +3684,11 @@
       <c r="H25" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I25" s="5" t="inlineStr"/>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>_cleanup_expired_sessions() with TTL=28800s. Lazy cleanup on access.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3648,7 +3740,11 @@
       <c r="H26" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>get_or_create_session() creates new executor on new session_id.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -3691,13 +3787,17 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>✅ Done</t>
+          <t>⚠️ Partial</t>
         </is>
       </c>
       <c r="H27" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I27" s="5" t="inlineStr"/>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>CLARIFICATION section in prompt template. Depends on config population.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3743,13 +3843,17 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>✅ Done</t>
+          <t>⚠️ Partial</t>
         </is>
       </c>
       <c r="H28" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>clarify_ambiguous_prompt config exists but defaults to empty string.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -3798,7 +3902,11 @@
       <c r="H29" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I29" s="5" t="inlineStr"/>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>_is_fallback_response() detects no-match. Retry + FAISS fallback.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3847,7 +3955,11 @@
       <c r="H30" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Safe fallback message returned. _direct_faiss_search() last resort.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -3900,7 +4012,11 @@
       <c r="H31" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I31" s="5" t="inlineStr"/>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>save_escalation() in escalation_store.py. _escalate() in agent.py. 11 tests in test_escalation.py (no AC tags).</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3954,7 +4070,11 @@
       <c r="H32" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>_notify_slack() webhook. Admin GET /admin/escalations. 11 tests (no AC tags).</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -4004,7 +4124,11 @@
       <c r="H33" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="I33" s="5" t="inlineStr"/>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>FORM GUIDANCE in agent_system_prompt. 6 AC-tagged tests.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4048,13 +4172,17 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Partial (AC4 blocked on UC-16)</t>
+          <t>⚠️ Partial</t>
         </is>
       </c>
       <c r="H34" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="I34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>FORM LOCATION GUIDANCE in prompt. AC4 blocked on UC-16. 5 AC-tagged tests.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -4101,9 +4229,13 @@
         </is>
       </c>
       <c r="H35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="5" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>workflow_guard.py detect_workflow_attempt(). 14 AC-tagged tests.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4152,9 +4284,13 @@
         </is>
       </c>
       <c r="H36" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" s="2" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Refusal in chat_router.py. Configurable message. 3 AC-tagged tests.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -4203,7 +4339,11 @@
       <c r="H37" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I37" s="5" t="inlineStr"/>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>IRRELEVANT QUERIES section in REACT_TEMPLATE prompt.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4253,7 +4393,11 @@
       <c r="H38" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Polite decline message configurable via irrelevant_query_response.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -4303,7 +4447,11 @@
       <c r="H39" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I39" s="5" t="inlineStr"/>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>guardrails.py Layer1 (patterns) + Layer2 (LLM). 27 tests in test_guardrails.py (no AC tags).</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4354,7 +4502,11 @@
       <c r="H40" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>GuardrailViolation → HTTP 400 + safe message in chat_router.py.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -4404,7 +4556,11 @@
       <c r="H41" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I41" s="5" t="inlineStr"/>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>Guardrail block logged to escalation_store via save_escalation().</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4453,7 +4609,11 @@
       <c r="H42" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>POST /feedback endpoint. FeedbackRequest with positive/negative rating. 12 tests (no AC tags).</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -4506,7 +4666,11 @@
       <c r="H43" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I43" s="5" t="inlineStr"/>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>comment field optional (default ''). Stored in DynamoDB.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4566,7 +4730,11 @@
       <c r="H44" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Roles hardcoded in models.py. No admin CRUD API. Gap M10.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -4629,7 +4797,11 @@
       <c r="H45" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I45" s="5" t="inlineStr"/>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>No connector config API. Only basic document upload.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4689,7 +4861,11 @@
       <c r="H46" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Only manual ingest endpoint. No scheduling/sync controls.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -4745,7 +4921,11 @@
       <c r="H47" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I47" s="5" t="inlineStr"/>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>No admin session management API.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4804,7 +4984,11 @@
       <c r="H48" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Fallback messages configurable via env vars only, not runtime admin API.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
@@ -4861,13 +5045,17 @@
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>❌ Pending</t>
+          <t>⚠️ Partial</t>
         </is>
       </c>
       <c r="H49" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I49" s="5" t="inlineStr"/>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>Escalations saved to DynamoDB + Slack webhook. No admin routing config UI.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4924,7 +5112,11 @@
       <c r="H50" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Frontend theme hardcoded. No admin theming API.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
@@ -5004,7 +5196,11 @@
       <c r="H51" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I51" s="5" t="inlineStr"/>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>No analytics endpoints or dashboard.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -5074,7 +5270,11 @@
       <c r="H52" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Only PDF accepted. No format toggle. Gap M9.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -5151,7 +5351,11 @@
       <c r="H53" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I53" s="5" t="inlineStr"/>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>No connector governance API.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>